<commit_message>
Atualiza planilha resumida do TBMT + Polvo (nova correção)
CAPEX "Em análise": Bravo inalterado (US$ 7,42 mi), Polvo A cai de
US$ 1,69 mi para US$ 1,65 mi (total US$ 9,07 mi). Recusadas: Bravo
cai de US$ 14,82 mi para US$ 14,33 mi (total US$ 18,13 mi). Apenas
CAPEX, sem Desenvolvimento de Produção. Totais conferidos contra a
aba Overview da fonte.
</commit_message>
<xml_diff>
--- a/Plano_Integrado_-_TBMTPOLVO_REV2_enxuta.xlsx
+++ b/Plano_Integrado_-_TBMTPOLVO_REV2_enxuta.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1177,21 +1177,21 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>43134.25</v>
+        <v>411880</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Medidor Coriolis - Separador de Teste</t>
+          <t>Novas Destiladoras</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1200,19 +1200,19 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>278926</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>71818</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>61136</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>43134.25</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1238,21 +1238,21 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>411880</v>
+        <v>50000</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Novas Destiladoras</t>
+          <t>NR-35 - Instalação das linhas de vida p/ escadas verticais e inspeção trava-quedas retrátil</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Bem Estar/Segurança</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1261,25 +1261,25 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>278926</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>71818</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>61136</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
@@ -1299,11 +1299,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>50000</v>
+        <v>150000</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1334,13 +1334,13 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>25000</v>
+        <v>150000</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
@@ -1360,7 +1360,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>150000</v>
+        <v>210000</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1369,12 +1369,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>NR-35 - Instalação das linhas de vida p/ escadas verticais e inspeção trava-quedas retrátil</t>
+          <t>NR13 - MBK-1130 (DEHYDRATOR) - AASJ &amp; INTERNOS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bem Estar/Segurança</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1392,16 +1392,16 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>105000</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>105000</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -1421,7 +1421,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>210000</v>
+        <v>300000</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>NR13 - MBK-1130 (DEHYDRATOR) - AASJ &amp; INTERNOS</t>
+          <t>NR13 - MBK-1130 (DEHYDRATOR) - IKM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1450,13 +1450,13 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="I17" t="n">
-        <v>105000</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>105000</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>300000</v>
+        <v>70000</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>NR13 - MBK-1130 (DEHYDRATOR) - IKM</t>
+          <t>NR13 - MBK-1130 (DEHYDRATOR) - VENDOR PINTURA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1511,13 +1511,13 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>300000</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>70000</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1543,21 +1543,21 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>70000</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>NR13 - MBK-1130 (DEHYDRATOR) - VENDOR PINTURA</t>
+          <t>PÓS TA - Andaime</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1578,7 +1578,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>70000</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1669,12 +1669,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PÓS TA - Andaime</t>
+          <t>PÓS TA - Caldeiraria</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1791,12 +1791,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PÓS TA - Caldeiraria</t>
+          <t>PÓS TA - Elétrica</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1913,12 +1913,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PÓS TA - Elétrica</t>
+          <t>PÓS TA - Mecânica</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2035,12 +2035,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PÓS TA - Mecânica</t>
+          <t>PÓS TA - NR13</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2157,12 +2157,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PÓS TA - NR13</t>
+          <t>PÓS TA - Pintura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2279,12 +2279,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PÓS TA - Pintura</t>
+          <t>PÓS TA - Supervisão - PRIO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2397,7 +2397,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2406,7 +2406,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PÓS TA - Supervisão - PRIO</t>
+          <t>Redundância do Sistema de Compressão de Gás - Trem Alfa + Trem Bravo</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2444,13 +2444,13 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="O33" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="Q33" t="n">
         <v>0</v>
@@ -2458,21 +2458,21 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>360000</v>
+        <v>609000</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Redundância do Sistema de Compressão de Gás - Trem Alfa + Trem Bravo</t>
+          <t>Retrofit do Motor - Bomba de Incêndio</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2496,7 +2496,7 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>609000</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -2505,13 +2505,13 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>120000</v>
+        <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>120000</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>120000</v>
+        <v>0</v>
       </c>
       <c r="Q34" t="n">
         <v>0</v>
@@ -2519,7 +2519,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>609000</v>
+        <v>544818</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2528,12 +2528,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Retrofit do Motor - Bomba de Incêndio</t>
+          <t>Revitalização do compressor de Ar de Instrumento</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2557,7 +2557,7 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>609000</v>
+        <v>0</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
@@ -2572,29 +2572,29 @@
         <v>0</v>
       </c>
       <c r="P35" t="n">
-        <v>0</v>
+        <v>341818</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
+        <v>203000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>544818</v>
+        <v>48096.59</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Revitalização do compressor de Ar de Instrumento</t>
+          <t>Vent de Químicos - Campanha 1/4</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Bem Estar/Segurança</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2612,7 +2612,7 @@
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>48096.59</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -2633,10 +2633,10 @@
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>341818</v>
+        <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>203000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Vent de Químicos - Campanha 1/4</t>
+          <t>Vent de Químicos - Campanha 2/4</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2673,10 +2673,10 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
         <v>48096.59</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Vent de Químicos - Campanha 2/4</t>
+          <t>Vent de Químicos - Campanha 3/4</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2737,10 +2737,10 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
         <v>48096.59</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0</v>
       </c>
       <c r="L38" t="n">
         <v>0</v>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Vent de Químicos - Campanha 3/4</t>
+          <t>Vent de Químicos - Campanha 4/4</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2801,11 +2801,11 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
         <v>48096.59</v>
       </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
       <c r="M39" t="n">
         <v>0</v>
       </c>
@@ -2819,67 +2819,6 @@
         <v>0</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>48096.59</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Vent de Químicos - Campanha 4/4</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Bem Estar/Segurança</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" t="n">
-        <v>0</v>
-      </c>
-      <c r="L40" t="n">
-        <v>48096.59</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0</v>
-      </c>
-      <c r="N40" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2894,7 +2833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q101"/>
+  <dimension ref="A1:Q93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3169,7 +3108,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>117516.57</v>
+        <v>28635.03</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -3178,7 +3117,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dehydrator - Revitalizacao - Reparo a bordo + comissionamento (SLB/Cameron)</t>
+          <t>Dehydrator - Revitalizacao - Survey interno (SLB/Cameron)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3192,7 +3131,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>28635.03</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -3207,10 +3146,10 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>88881.53999999999</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>28635.03</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -3230,16 +3169,16 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>28635.03</v>
+        <v>120000</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dehydrator - Revitalizacao - Survey interno (SLB/Cameron)</t>
+          <t>ESTUDO DE ENGENHARIA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -3253,54 +3192,54 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>28635.03</v>
+        <v>10000</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>120000</v>
+        <v>239673.08</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ESTUDO DE ENGENHARIA</t>
+          <t>Filtros na Entrada da Água do Mar do Vacuum Condenser - instalação de novos filtros</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3314,45 +3253,45 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>10000</v>
+        <v>119836.54</v>
       </c>
       <c r="N7" t="n">
-        <v>10000</v>
+        <v>119836.54</v>
       </c>
       <c r="O7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>239673.08</v>
+        <v>96153.84</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -3361,12 +3300,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Filtros na Entrada da Água do Mar do Vacuum Condenser - instalação de novos filtros</t>
+          <t>GTG - Melhoria lavagem turbina, aquecimento da água</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3396,10 +3335,10 @@
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>119836.54</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>119836.54</v>
+        <v>96153.84</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -3413,7 +3352,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>96153.84</v>
+        <v>180000</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -3422,12 +3361,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GTG - Melhoria lavagem turbina, aquecimento da água</t>
+          <t>GTG - Monitoramento Remoto Baker</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3457,10 +3396,10 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>180000</v>
       </c>
       <c r="N9" t="n">
-        <v>96153.84</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -3474,7 +3413,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>180000</v>
+        <v>97191.46000000001</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -3483,12 +3422,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GTG - Monitoramento Remoto Baker</t>
+          <t>GTG - Sistema de Lubrificação dedicado (MLO)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3512,13 +3451,13 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>97191.46000000001</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>180000</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -3535,7 +3474,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>97191.46000000001</v>
+        <v>162218.61</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -3544,7 +3483,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GTG - Sistema de Lubrificação dedicado (MLO)</t>
+          <t>GTG - Sistema de Lubrificação dedicado (Partida &amp; SLO)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3573,7 +3512,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>97191.46000000001</v>
+        <v>162218.61</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -3596,21 +3535,21 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>162218.61</v>
+        <v>38167.94</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GTG - Sistema de Lubrificação dedicado (Partida &amp; SLO)</t>
+          <t>ID- 001 Continuidade comunicação vaso - ABB - PI</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3625,7 +3564,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>38167.94</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -3634,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>162218.61</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -3657,7 +3596,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>341836.62</v>
+        <v>100455.91</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -3666,7 +3605,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Heat Tracing - Finalização do serviço</t>
+          <t>ID- 001 Instalação computador de vazão ROC</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -3686,7 +3625,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>100455.91</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -3713,21 +3652,21 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>341836.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>38167.94</v>
+        <v>14350.76</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ID- 001 Continuidade comunicação vaso - ABB - PI</t>
+          <t>ID- 001 Survey Instalação computador de vazão ROC</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -3744,10 +3683,10 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>14350.76</v>
       </c>
       <c r="H14" t="n">
-        <v>38167.94</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -3779,7 +3718,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>100455.91</v>
+        <v>172209.92</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -3788,7 +3727,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ID- 001 Instalação computador de vazão ROC</t>
+          <t>ID- 001 Validação Instalação computador de vazão ROC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3808,10 +3747,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>100455.91</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>172209.92</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -3840,7 +3779,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14350.76</v>
+        <v>226198.66</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -3849,7 +3788,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ID- 001 Survey Instalação computador de vazão ROC</t>
+          <t>ID- 002  Validação Adequação sistema supervisório de medição - FASE 2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -3866,7 +3805,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>14350.76</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -3896,12 +3835,12 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>226198.66</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>172209.92</v>
+        <v>60859.92</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -3910,7 +3849,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ID- 001 Validação Instalação computador de vazão ROC</t>
+          <t>ID- 002 Survey Adequação sistema supervisório de medição - FASE 1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -3924,7 +3863,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>60859.92</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -3933,7 +3872,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>172209.92</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -3962,7 +3901,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>226198.66</v>
+        <v>16698.47</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -3971,7 +3910,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ID- 002  Validação Adequação sistema supervisório de medição - FASE 2</t>
+          <t>ID- 003 Adequações topside -  Autorização de uso - troca turbina por coriolis -1198A</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -3988,7 +3927,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>16698.47</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -4018,12 +3957,12 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>226198.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>60859.92</v>
+        <v>16698.48</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -4032,7 +3971,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ID- 002 Survey Adequação sistema supervisório de medição - FASE 1</t>
+          <t>ID- 003 Adequações topside -  Autorização de uso - troca turbina por coriolis -1198B</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -4046,7 +3985,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>60859.92</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -4058,7 +3997,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>16698.48</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -4084,7 +4023,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>16698.47</v>
+        <v>22900.76</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -4093,7 +4032,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ID- 003 Adequações topside -  Autorização de uso - troca turbina por coriolis -1198A</t>
+          <t>ID- 003 Embarque ANP - Autorização de uso - troca turbina por coriolis -1198A</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -4110,7 +4049,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>16698.47</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -4122,7 +4061,7 @@
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>22900.76</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -4145,7 +4084,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>16698.48</v>
+        <v>22900.76</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -4154,7 +4093,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ID- 003 Adequações topside -  Autorização de uso - troca turbina por coriolis -1198B</t>
+          <t>ID- 003 Embarque ANP - Autorização de uso - troca turbina por coriolis -1198A</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -4180,7 +4119,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>16698.48</v>
+        <v>22900.76</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -4206,7 +4145,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>22900.76</v>
+        <v>6297.71</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -4215,7 +4154,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ID- 003 Embarque ANP - Autorização de uso - troca turbina por coriolis -1198A</t>
+          <t>ID- 003 Survey - validação de material - Autorização de uso - troca turbina por coriolis</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4232,7 +4171,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>6297.71</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -4244,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>22900.76</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -4267,7 +4206,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22900.76</v>
+        <v>19047.62</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -4276,7 +4215,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ID- 003 Embarque ANP - Autorização de uso - troca turbina por coriolis -1198A</t>
+          <t>ID- 004 Instalação - Adequação dos pontos de amostragem - Fuel gás + Separador teste</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -4296,13 +4235,13 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>19047.62</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>22900.76</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -4328,7 +4267,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>6297.71</v>
+        <v>6285.72</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -4337,7 +4276,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ID- 003 Survey - validação de material - Autorização de uso - troca turbina por coriolis</t>
+          <t xml:space="preserve">ID- 004 Survey - validação de material - Adequação dos pontos de amostragem - Fuel gás + Separador teste </t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -4354,7 +4293,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>6297.71</v>
+        <v>6285.72</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -4389,7 +4328,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>19047.62</v>
+        <v>11428.57</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -4398,7 +4337,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ID- 004 Instalação - Adequação dos pontos de amostragem - Fuel gás + Separador teste</t>
+          <t xml:space="preserve">ID- 005 Instalação - misturador estático </t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -4418,7 +4357,7 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>19047.62</v>
+        <v>11428.57</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -4450,7 +4389,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>6285.72</v>
+        <v>1428.57</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -4459,7 +4398,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID- 004 Survey - validação de material - Adequação dos pontos de amostragem - Fuel gás + Separador teste </t>
+          <t xml:space="preserve">ID- 005 Survey - validação de material- Instalação misturador estático </t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -4476,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>6285.72</v>
+        <v>1428.57</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -4511,7 +4450,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>11428.57</v>
+        <v>104761.9</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -4520,7 +4459,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID- 005 Instalação - misturador estático </t>
+          <t>ID- 007 Readequação comunicação Intouch e Focqus</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -4540,10 +4479,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>11428.57</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>104761.9</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -4572,21 +4511,21 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1428.57</v>
+        <v>150000</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID- 005 Survey - validação de material- Instalação misturador estático </t>
+          <t>Implantação do projeto 'Muster Digital'</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Bem Estar/Segurança</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4598,7 +4537,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>1428.57</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -4622,7 +4561,7 @@
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -4633,7 +4572,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>104761.9</v>
+        <v>140000</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -4642,12 +4581,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ID- 007 Readequação comunicação Intouch e Focqus</t>
+          <t>Implantação do projeto 'Muster Digital'</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Bem Estar/Segurança</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -4665,7 +4604,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>104761.9</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -4686,7 +4625,7 @@
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>140000</v>
       </c>
       <c r="Q29" t="n">
         <v>0</v>
@@ -4694,21 +4633,21 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>150000</v>
+        <v>49813</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Implantação do projeto 'Muster Digital'</t>
+          <t>Instalação de um equipamento de içamento de carga na casa de bombas</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Bem Estar/Segurança</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -4738,13 +4677,13 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>49813</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
@@ -4755,7 +4694,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>140000</v>
+        <v>19226.08</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -4764,12 +4703,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Implantação do projeto 'Muster Digital'</t>
+          <t>Linha de Reprocessamento do Separador de Teste - Survey e delineamento (RADIX)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bem Estar/Segurança</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -4784,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>19226.08</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -4808,7 +4747,7 @@
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>140000</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="n">
         <v>0</v>
@@ -4816,7 +4755,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>49813</v>
+        <v>38095.24</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -4825,12 +4764,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Instalação de um equipamento de içamento de carga na casa de bombas</t>
+          <t>Medição virtual + Consultoria Solution Seeker</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -4860,7 +4799,7 @@
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>49813</v>
+        <v>0</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
@@ -4872,21 +4811,21 @@
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
+        <v>38095.24</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>19226.08</v>
+        <v>162085.78</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Linha de Reprocessamento do Separador de Teste - Survey e delineamento (RADIX)</t>
+          <t>Mobilização TA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4900,13 +4839,13 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>162085.78</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>19226.08</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -4938,21 +4877,21 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>38095.24</v>
+        <v>519230.77</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Medição virtual + Consultoria Solution Seeker</t>
+          <t>MPP - Adequação do sistema de Selagem Multifásica</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4973,7 +4912,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>519230.77</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -4994,12 +4933,12 @@
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>38095.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>162085.78</v>
+        <v>50909.09</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -5008,12 +4947,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mobilização TA</t>
+          <t>Obstrução Sistema de Águas Cinzas</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5022,7 +4961,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>162085.78</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -5046,7 +4985,7 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>0</v>
+        <v>50909.09</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
@@ -5060,7 +4999,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>519230.77</v>
+        <v>20647.06</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -5069,12 +5008,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MPP - Adequação do sistema de Selagem Multifásica</t>
+          <t>Polvo-A - Novos Sistemas de Dosagem Química - Flow Improver + Inibidor de Corrosão</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -5092,10 +5031,10 @@
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>20647.06</v>
       </c>
       <c r="J36" t="n">
-        <v>519230.77</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -5121,7 +5060,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>50909.09</v>
+        <v>29911.62</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -5130,12 +5069,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Obstrução Sistema de Águas Cinzas</t>
+          <t>Polvo-A - Sistema de Químicos - Survey as-found prévio à modificação das bombas (RADIX)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5144,7 +5083,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>29911.62</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -5168,7 +5107,7 @@
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>50909.09</v>
+        <v>0</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -5182,7 +5121,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0</v>
+        <v>32256.45454545454</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -5191,7 +5130,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Polvo-A - Novo Compressor de Ar de Instrumento - acompanhamento do projeto</t>
+          <t>PRÉ TA - Andaime</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -5205,7 +5144,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>32256.45454545454</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -5243,16 +5182,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0</v>
+        <v>70743.8</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Polvo-A - Novo Separador de Teste</t>
+          <t>PRÉ TA - Andaime</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5266,7 +5205,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>70743.8</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -5304,7 +5243,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>20647.06</v>
+        <v>132884.9175709091</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -5313,7 +5252,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Polvo-A - Novos Sistemas de Dosagem Química - Flow Improver + Inibidor de Corrosão</t>
+          <t>PRÉ TA - Caldeiraria</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -5327,7 +5266,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>132884.9175709091</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -5336,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>20647.06</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -5365,16 +5304,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0</v>
+        <v>67152.94516363635</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Polvo-A - Sistema de Medição Multifásica na Linha de Exportação</t>
+          <t>PRÉ TA - Caldeiraria</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5388,7 +5327,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>67152.94516363635</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -5426,7 +5365,7 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>29911.62</v>
+        <v>4000</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -5435,7 +5374,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Polvo-A - Sistema de Químicos - Survey as-found prévio à modificação das bombas (RADIX)</t>
+          <t>PRÉ TA - Elétrica</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5449,7 +5388,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>29911.62</v>
+        <v>4000</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
@@ -5487,16 +5426,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>32256.45454545454</v>
+        <v>22000</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PRÉ TA - Andaime</t>
+          <t>PRÉ TA - Elétrica</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5510,7 +5449,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>32256.45454545454</v>
+        <v>22000</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -5548,16 +5487,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>70743.8</v>
+        <v>5000</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PRÉ TA - Andaime</t>
+          <t>PRÉ TA - Mecânica</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5571,7 +5510,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>70743.8</v>
+        <v>5000</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
@@ -5609,16 +5548,16 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>132884.9175709091</v>
+        <v>18000</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PRÉ TA - Caldeiraria</t>
+          <t>PRÉ TA - Mecânica</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5632,7 +5571,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>132884.9175709091</v>
+        <v>18000</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -5670,16 +5609,16 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>67152.94516363635</v>
+        <v>65060</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PRÉ TA - Caldeiraria</t>
+          <t>PRÉ TA - NR13</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5693,7 +5632,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>67152.94516363635</v>
+        <v>65060</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
@@ -5731,16 +5670,16 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>4000</v>
+        <v>130715</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PRÉ TA - Elétrica</t>
+          <t>PRÉ TA - NR13</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5754,7 +5693,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>4000</v>
+        <v>130715</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -5792,16 +5731,16 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>22000</v>
+        <v>0</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PRÉ TA - Elétrica</t>
+          <t>PRÉ TA - Supervisão - PRIO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5815,7 +5754,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>22000</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -5853,16 +5792,16 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PRÉ TA - Mecânica</t>
+          <t>PRÉ TA - Supervisão - PRIO</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5876,7 +5815,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
@@ -5914,7 +5853,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>18000</v>
+        <v>0</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -5923,7 +5862,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PRÉ TA - Mecânica</t>
+          <t>Redundância Trocador de Calor do Compressor</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5937,7 +5876,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>18000</v>
+        <v>0</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -5975,7 +5914,7 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>65060</v>
+        <v>298000</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -5984,12 +5923,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PRÉ TA - NR13</t>
+          <t>Reforma dos banheiros dos camarotes de POLVO A</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -5998,16 +5937,16 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>65060</v>
+        <v>85000</v>
       </c>
       <c r="G51" t="n">
-        <v>0</v>
+        <v>155000</v>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>28000</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -6036,16 +5975,16 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>130715</v>
+        <v>217881</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>PRÉ TA - NR13</t>
+          <t>Repetidoras de Rádio</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6059,7 +5998,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>130715</v>
+        <v>0</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
@@ -6068,7 +6007,7 @@
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>217881</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -6097,21 +6036,21 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>0</v>
+        <v>170000</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PRÉ TA - Pintura</t>
+          <t xml:space="preserve">Retrofit sistema fixo de CO2 </t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Bem Estar/Segurança</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -6132,7 +6071,7 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>170000</v>
       </c>
       <c r="K53" t="n">
         <v>0</v>
@@ -6158,7 +6097,7 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0</v>
+        <v>687000</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -6167,12 +6106,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>PRÉ TA - Pintura</t>
+          <t>REVAMP CARGO PUMP - Nº 2</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -6205,7 +6144,7 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0</v>
+        <v>687000</v>
       </c>
       <c r="O54" t="n">
         <v>0</v>
@@ -6219,21 +6158,21 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0</v>
+        <v>721903</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PRÉ TA - Supervisão - PRIO</t>
+          <t>REVAMP CARGO PUMP - Nº 2</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -6266,7 +6205,7 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>721903</v>
       </c>
       <c r="O55" t="n">
         <v>0</v>
@@ -6280,7 +6219,7 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>0</v>
+        <v>57342.75</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -6289,12 +6228,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PRÉ TA - Supervisão - PRIO</t>
+          <t>Revitalização do Sistema de Tratamento do Slop - Survey as-found (SLB)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -6309,7 +6248,7 @@
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>0</v>
+        <v>57342.75</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
@@ -6341,7 +6280,7 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0</v>
+        <v>209580</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -6350,12 +6289,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Redundância Trocador de Calor do Compressor</t>
+          <t>Saneamento de backlog de as built de MOCs</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -6364,59 +6303,59 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="M57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="O57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>17465</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>298000</v>
+        <v>705900</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Reforma dos banheiros dos camarotes de POLVO A</t>
+          <t>Sistema de Cloração - 2 unidades Chloropac SB3K + implantação</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -6425,16 +6364,16 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>85000</v>
+        <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>155000</v>
+        <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>28000</v>
+        <v>0</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -6458,26 +6397,26 @@
         <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>705900</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>217881</v>
+        <v>79049.33</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Repetidoras de Rádio</t>
+          <t>Sistema de Cloração / Eletrocloradora - Survey as-found e delineamento (RADIX)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6492,10 +6431,10 @@
         <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>79049.33</v>
       </c>
       <c r="I59" t="n">
-        <v>217881</v>
+        <v>0</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
@@ -6524,21 +6463,21 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>170000</v>
+        <v>18390.25454545455</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retrofit sistema fixo de CO2 </t>
+          <t>TA - Andaime</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Bem Estar/Segurança</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -6547,7 +6486,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0</v>
+        <v>18390.25454545455</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -6559,7 +6498,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>170000</v>
+        <v>0</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -6585,7 +6524,7 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>687000</v>
+        <v>25266</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -6594,12 +6533,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>REVAMP CARGO PUMP - Nº 2</t>
+          <t>TA - Andaime</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -6608,7 +6547,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>0</v>
+        <v>25266</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -6632,7 +6571,7 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>687000</v>
+        <v>0</v>
       </c>
       <c r="O61" t="n">
         <v>0</v>
@@ -6646,21 +6585,21 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>721903</v>
+        <v>484883.4333090909</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>REVAMP CARGO PUMP - Nº 2</t>
+          <t>TA - Caldeiraria</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -6669,7 +6608,7 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
+        <v>484883.4333090909</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
@@ -6693,7 +6632,7 @@
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>721903</v>
+        <v>0</v>
       </c>
       <c r="O62" t="n">
         <v>0</v>
@@ -6707,7 +6646,7 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>57342.75</v>
+        <v>816120</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -6716,12 +6655,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Revitalização do Sistema de Tratamento do Slop - Survey as-found (SLB)</t>
+          <t>TA - Caldeiraria</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -6730,13 +6669,13 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>816120</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>57342.75</v>
+        <v>0</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
@@ -6768,16 +6707,16 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>209580</v>
+        <v>526122.67</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Saneamento de backlog de as built de MOCs</t>
+          <t>TA - Compra de Placas de controle dos VFDs Rockwell</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -6791,59 +6730,59 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>17465</v>
+        <v>526122.67</v>
       </c>
       <c r="G64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="H64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="K64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="L64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="M64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
       <c r="Q64" t="n">
-        <v>17465</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>705900</v>
+        <v>162085.78</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Sistema de Cloração - 2 unidades Chloropac SB3K + implantação</t>
+          <t>TA - Desmobilização</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -6855,7 +6794,7 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>162085.78</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -6885,12 +6824,12 @@
         <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>705900</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>79049.33</v>
+        <v>247572.33</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -6899,12 +6838,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Sistema de Cloração / Eletrocloradora - Survey as-found e delineamento (RADIX)</t>
+          <t>TA - Desmobilização</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -6916,10 +6855,10 @@
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>247572.33</v>
       </c>
       <c r="H66" t="n">
-        <v>79049.33</v>
+        <v>0</v>
       </c>
       <c r="I66" t="n">
         <v>0</v>
@@ -6951,16 +6890,16 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>29911.62</v>
+        <v>52427</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Sistema de Quimicos (Novas Bombas) - Survey as-found e mapeamento da revitalizacao (RADIX)</t>
+          <t>TA - Elétrica</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -6974,10 +6913,10 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0</v>
+        <v>52427</v>
       </c>
       <c r="G67" t="n">
-        <v>29911.62</v>
+        <v>0</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -7012,16 +6951,16 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>18390.25454545455</v>
+        <v>982417</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>TA - Andaime</t>
+          <t>TA - Elétrica</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7035,7 +6974,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>18390.25454545455</v>
+        <v>982417</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
@@ -7073,7 +7012,7 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>25266</v>
+        <v>107277.79</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -7082,12 +7021,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>TA - Andaime</t>
+          <t>TA - Ensaios Avançados</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -7096,7 +7035,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>25266</v>
+        <v>107277.79</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
@@ -7134,7 +7073,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>484883.4333090909</v>
+        <v>206792.87</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -7143,12 +7082,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>TA - Caldeiraria</t>
+          <t>TA - Flowline - Passagem de PIG</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -7157,7 +7096,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>484883.4333090909</v>
+        <v>206792.87</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -7195,7 +7134,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>816120</v>
+        <v>16775</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -7204,12 +7143,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>TA - Caldeiraria</t>
+          <t>TA - Ignitor do Flare</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -7218,7 +7157,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>816120</v>
+        <v>16775</v>
       </c>
       <c r="G71" t="n">
         <v>0</v>
@@ -7256,16 +7195,16 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>526122.67</v>
+        <v>214491.29</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>TA - Compra de Placas de controle dos VFDs Rockwell</t>
+          <t>TA - Manutenção no Swivel elétrico</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7279,7 +7218,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>526122.67</v>
+        <v>214491.29</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
@@ -7317,21 +7256,21 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>162085.78</v>
+        <v>105384.62</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TA - Desmobilização</t>
+          <t>TA - Manutenção Preventiva de Painéis ABB</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -7340,10 +7279,10 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>0</v>
+        <v>105384.62</v>
       </c>
       <c r="G73" t="n">
-        <v>162085.78</v>
+        <v>0</v>
       </c>
       <c r="H73" t="n">
         <v>0</v>
@@ -7378,7 +7317,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>247572.33</v>
+        <v>128019.23</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -7387,12 +7326,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>TA - Desmobilização</t>
+          <t>TA - Manutenção Preventiva dos VFDs Innomotics</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -7401,10 +7340,10 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
+        <v>128019.23</v>
       </c>
       <c r="G74" t="n">
-        <v>247572.33</v>
+        <v>0</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
@@ -7439,7 +7378,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>52427</v>
+        <v>114769.62</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -7448,12 +7387,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>TA - Elétrica</t>
+          <t>TA - Manutenção Preventiva dos VFDs Rockwell</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -7462,7 +7401,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>52427</v>
+        <v>114769.62</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -7500,16 +7439,16 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>982417</v>
+        <v>76237</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>TA - Elétrica</t>
+          <t>TA - Mecânica</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7523,7 +7462,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>982417</v>
+        <v>76237</v>
       </c>
       <c r="G76" t="n">
         <v>0</v>
@@ -7561,7 +7500,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>107277.79</v>
+        <v>1478997</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -7570,12 +7509,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>TA - Ensaios Avançados</t>
+          <t>TA - Mecânica</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -7584,7 +7523,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>107277.79</v>
+        <v>1478997</v>
       </c>
       <c r="G77" t="n">
         <v>0</v>
@@ -7622,21 +7561,21 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>206792.87</v>
+        <v>247572.33</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>TA - Flowline - Passagem de PIG</t>
+          <t>TA - Mobilização</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7645,10 +7584,10 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>206792.87</v>
+        <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>0</v>
+        <v>247572.33</v>
       </c>
       <c r="H78" t="n">
         <v>0</v>
@@ -7683,7 +7622,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>16775</v>
+        <v>134009</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -7692,12 +7631,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>TA - Ignitor do Flare</t>
+          <t>TA - Monitoramento da Qualidade de Energia - BCS</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Integridade e Regulatório</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -7706,7 +7645,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>16775</v>
+        <v>134009</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -7744,21 +7683,21 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>214491.29</v>
+        <v>173229.0588235294</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TA - Manutenção no Swivel elétrico</t>
+          <t>TA - NR13</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7767,7 +7706,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>214491.29</v>
+        <v>173229.0588235294</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
@@ -7805,7 +7744,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>105384.62</v>
+        <v>659418</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -7814,12 +7753,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>TA - Manutenção Preventiva de Painéis ABB</t>
+          <t>TA - NR13</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7828,7 +7767,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>105384.62</v>
+        <v>659418</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -7866,21 +7805,21 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>128019.23</v>
+        <v>29414.94545454545</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>TA - Manutenção Preventiva dos VFDs Innomotics</t>
+          <t>TA - Pintura</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7889,7 +7828,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>128019.23</v>
+        <v>29414.94545454545</v>
       </c>
       <c r="G82" t="n">
         <v>0</v>
@@ -7927,21 +7866,21 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>114769.62</v>
+        <v>53415</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>TA - Manutenção Preventiva dos VFDs Rockwell</t>
+          <t>TA - Pintura</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Rotina Operacional</t>
+          <t>Eficiência de Produção</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7950,7 +7889,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>114769.62</v>
+        <v>53415</v>
       </c>
       <c r="G83" t="n">
         <v>0</v>
@@ -7988,7 +7927,7 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>76237</v>
+        <v>0</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -7997,7 +7936,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>TA - Mecânica</t>
+          <t>TA - Supervisão - PRIO</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -8011,7 +7950,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>76237</v>
+        <v>0</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
@@ -8049,7 +7988,7 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1478997</v>
+        <v>0</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -8058,7 +7997,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>TA - Mecânica</t>
+          <t>TA - Supervisão - PRIO</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8072,7 +8011,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>1478997</v>
+        <v>0</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
@@ -8110,7 +8049,7 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>247572.33</v>
+        <v>1399134.41</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -8119,12 +8058,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>TA - Mobilização</t>
+          <t>TA - Swivel - Pacote Hidráulico (OneSubsea)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -8133,10 +8072,10 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0</v>
+        <v>1399134.41</v>
       </c>
       <c r="G86" t="n">
-        <v>247572.33</v>
+        <v>0</v>
       </c>
       <c r="H86" t="n">
         <v>0</v>
@@ -8171,7 +8110,7 @@
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>134009</v>
+        <v>102166.41</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -8180,7 +8119,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>TA - Monitoramento da Qualidade de Energia - BCS</t>
+          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 1/4</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -8194,7 +8133,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>134009</v>
+        <v>102166.41</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -8232,16 +8171,16 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>173229.0588235294</v>
+        <v>102166.41</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>TA - NR13</t>
+          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 2/4</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -8255,10 +8194,10 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>173229.0588235294</v>
+        <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>0</v>
+        <v>102166.41</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
@@ -8293,7 +8232,7 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>659418</v>
+        <v>102166.41</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -8302,7 +8241,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>TA - NR13</t>
+          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 3/4</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -8316,13 +8255,13 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>659418</v>
+        <v>0</v>
       </c>
       <c r="G89" t="n">
         <v>0</v>
       </c>
       <c r="H89" t="n">
-        <v>0</v>
+        <v>102166.41</v>
       </c>
       <c r="I89" t="n">
         <v>0</v>
@@ -8354,16 +8293,16 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>29414.94545454545</v>
+        <v>102166.41</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>TA - Pintura</t>
+          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 4/4</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8377,7 +8316,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>29414.94545454545</v>
+        <v>0</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -8386,7 +8325,7 @@
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>0</v>
+        <v>102166.41</v>
       </c>
       <c r="J90" t="n">
         <v>0</v>
@@ -8415,21 +8354,21 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>53415</v>
+        <v>105000</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
+          <t>Polvo A (Polvo Field)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>TA - Pintura</t>
+          <t>Troca da Estação Meteorológica</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Integridade e Regulatório</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -8438,13 +8377,13 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>53415</v>
+        <v>0</v>
       </c>
       <c r="G91" t="n">
         <v>0</v>
       </c>
       <c r="H91" t="n">
-        <v>0</v>
+        <v>105000</v>
       </c>
       <c r="I91" t="n">
         <v>0</v>
@@ -8476,21 +8415,21 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0</v>
+        <v>326923.08</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Polvo A (Polvo Field)</t>
+          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>TA - Supervisão - PRIO</t>
+          <t>Troca de bomba nacionalização das bombas críticas da praça de máquinas (Main cooling sea water, bomba de condensado e GS pump)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -8499,7 +8438,7 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>0</v>
+        <v>326923.08</v>
       </c>
       <c r="G92" t="n">
         <v>0</v>
@@ -8537,7 +8476,7 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>0</v>
+        <v>1710000</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -8546,12 +8485,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>TA - Supervisão - PRIO</t>
+          <t>Upgrade metering de gás e Diesel- GTGs</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Eficiência de Produção</t>
+          <t>Rotina Operacional</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -8593,494 +8532,6 @@
         <v>0</v>
       </c>
       <c r="Q93" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="n">
-        <v>1399134.41</v>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>TA - Swivel - Pacote Hidráulico (OneSubsea)</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Integridade e Regulatório</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F94" t="n">
-        <v>1399134.41</v>
-      </c>
-      <c r="G94" t="n">
-        <v>0</v>
-      </c>
-      <c r="H94" t="n">
-        <v>0</v>
-      </c>
-      <c r="I94" t="n">
-        <v>0</v>
-      </c>
-      <c r="J94" t="n">
-        <v>0</v>
-      </c>
-      <c r="K94" t="n">
-        <v>0</v>
-      </c>
-      <c r="L94" t="n">
-        <v>0</v>
-      </c>
-      <c r="M94" t="n">
-        <v>0</v>
-      </c>
-      <c r="N94" t="n">
-        <v>0</v>
-      </c>
-      <c r="O94" t="n">
-        <v>0</v>
-      </c>
-      <c r="P94" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q94" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 1/4</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>Eficiência de Produção</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F95" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="G95" t="n">
-        <v>0</v>
-      </c>
-      <c r="H95" t="n">
-        <v>0</v>
-      </c>
-      <c r="I95" t="n">
-        <v>0</v>
-      </c>
-      <c r="J95" t="n">
-        <v>0</v>
-      </c>
-      <c r="K95" t="n">
-        <v>0</v>
-      </c>
-      <c r="L95" t="n">
-        <v>0</v>
-      </c>
-      <c r="M95" t="n">
-        <v>0</v>
-      </c>
-      <c r="N95" t="n">
-        <v>0</v>
-      </c>
-      <c r="O95" t="n">
-        <v>0</v>
-      </c>
-      <c r="P95" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q95" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 2/4</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>Eficiência de Produção</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F96" t="n">
-        <v>0</v>
-      </c>
-      <c r="G96" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="H96" t="n">
-        <v>0</v>
-      </c>
-      <c r="I96" t="n">
-        <v>0</v>
-      </c>
-      <c r="J96" t="n">
-        <v>0</v>
-      </c>
-      <c r="K96" t="n">
-        <v>0</v>
-      </c>
-      <c r="L96" t="n">
-        <v>0</v>
-      </c>
-      <c r="M96" t="n">
-        <v>0</v>
-      </c>
-      <c r="N96" t="n">
-        <v>0</v>
-      </c>
-      <c r="O96" t="n">
-        <v>0</v>
-      </c>
-      <c r="P96" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q96" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 3/4</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Eficiência de Produção</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F97" t="n">
-        <v>0</v>
-      </c>
-      <c r="G97" t="n">
-        <v>0</v>
-      </c>
-      <c r="H97" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="I97" t="n">
-        <v>0</v>
-      </c>
-      <c r="J97" t="n">
-        <v>0</v>
-      </c>
-      <c r="K97" t="n">
-        <v>0</v>
-      </c>
-      <c r="L97" t="n">
-        <v>0</v>
-      </c>
-      <c r="M97" t="n">
-        <v>0</v>
-      </c>
-      <c r="N97" t="n">
-        <v>0</v>
-      </c>
-      <c r="O97" t="n">
-        <v>0</v>
-      </c>
-      <c r="P97" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q97" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Trem Bravo - Limpeza Crude-Crude + Crude Heater (IKM) - Campanha 4/4</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Eficiência de Produção</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F98" t="n">
-        <v>0</v>
-      </c>
-      <c r="G98" t="n">
-        <v>0</v>
-      </c>
-      <c r="H98" t="n">
-        <v>0</v>
-      </c>
-      <c r="I98" t="n">
-        <v>102166.41</v>
-      </c>
-      <c r="J98" t="n">
-        <v>0</v>
-      </c>
-      <c r="K98" t="n">
-        <v>0</v>
-      </c>
-      <c r="L98" t="n">
-        <v>0</v>
-      </c>
-      <c r="M98" t="n">
-        <v>0</v>
-      </c>
-      <c r="N98" t="n">
-        <v>0</v>
-      </c>
-      <c r="O98" t="n">
-        <v>0</v>
-      </c>
-      <c r="P98" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q98" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>105000</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Polvo A (Polvo Field)</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Troca da Estação Meteorológica</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Integridade e Regulatório</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F99" t="n">
-        <v>0</v>
-      </c>
-      <c r="G99" t="n">
-        <v>0</v>
-      </c>
-      <c r="H99" t="n">
-        <v>105000</v>
-      </c>
-      <c r="I99" t="n">
-        <v>0</v>
-      </c>
-      <c r="J99" t="n">
-        <v>0</v>
-      </c>
-      <c r="K99" t="n">
-        <v>0</v>
-      </c>
-      <c r="L99" t="n">
-        <v>0</v>
-      </c>
-      <c r="M99" t="n">
-        <v>0</v>
-      </c>
-      <c r="N99" t="n">
-        <v>0</v>
-      </c>
-      <c r="O99" t="n">
-        <v>0</v>
-      </c>
-      <c r="P99" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q99" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>326923.08</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Troca de bomba nacionalização das bombas críticas da praça de máquinas (Main cooling sea water, bomba de condensado e GS pump)</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Rotina Operacional</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F100" t="n">
-        <v>326923.08</v>
-      </c>
-      <c r="G100" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" t="n">
-        <v>0</v>
-      </c>
-      <c r="I100" t="n">
-        <v>0</v>
-      </c>
-      <c r="J100" t="n">
-        <v>0</v>
-      </c>
-      <c r="K100" t="n">
-        <v>0</v>
-      </c>
-      <c r="L100" t="n">
-        <v>0</v>
-      </c>
-      <c r="M100" t="n">
-        <v>0</v>
-      </c>
-      <c r="N100" t="n">
-        <v>0</v>
-      </c>
-      <c r="O100" t="n">
-        <v>0</v>
-      </c>
-      <c r="P100" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q100" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>1710000</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FPSO Bravo (TBMT Field) </t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Upgrade metering de gás e Diesel- GTGs</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Rotina Operacional</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="F101" t="n">
-        <v>0</v>
-      </c>
-      <c r="G101" t="n">
-        <v>0</v>
-      </c>
-      <c r="H101" t="n">
-        <v>0</v>
-      </c>
-      <c r="I101" t="n">
-        <v>0</v>
-      </c>
-      <c r="J101" t="n">
-        <v>0</v>
-      </c>
-      <c r="K101" t="n">
-        <v>0</v>
-      </c>
-      <c r="L101" t="n">
-        <v>0</v>
-      </c>
-      <c r="M101" t="n">
-        <v>0</v>
-      </c>
-      <c r="N101" t="n">
-        <v>0</v>
-      </c>
-      <c r="O101" t="n">
-        <v>0</v>
-      </c>
-      <c r="P101" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q101" t="n">
         <v>1710000</v>
       </c>
     </row>

</xml_diff>